<commit_message>
Mapa del predio en la home + stands reales
- Mapa del predio: SVG clickeable (VenueMap) redibujado del plano oficial
  (data-src/plano-predio.png). Cada stand → /stand/<id>; patios de comida y
  zonas de servicio como referencia no clickeable. Layout en src/config/venue.ts.
  Va en la home (sección "Mapa del predio"), con scroll horizontal para el
  teléfono. Flag FEATURES.mapa para prender/apagar.
- Stands reales del evento en data-src/stands.csv y stands.xlsx (52 stands de
  productos, 1–51 y 56; los 52–55 son patio de comidas y no van como stands).
  Reemplazan los datos de ejemplo. NOTA: no se regeneró public/data para no
  pisar los datos ya cargados; aplicar corriendo la ingesta cuando estén los
  productos reales.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZVuJK6DwE7KYatdvxUDTj
</commit_message>
<xml_diff>
--- a/data-src/stands.xlsx
+++ b/data-src/stands.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="105">
   <si>
     <t>Stand</t>
   </si>
@@ -19,184 +19,313 @@
     <t>Proveedor</t>
   </si>
   <si>
-    <t>Laboratorios Andino</t>
-  </si>
-  <si>
-    <t>Laboratorios Austral</t>
-  </si>
-  <si>
-    <t>Laboratorios del Plata</t>
-  </si>
-  <si>
-    <t>Laboratorios Pampa Sur</t>
-  </si>
-  <si>
-    <t>Laboratorios Cuyo</t>
-  </si>
-  <si>
-    <t>Laboratorios Litoral</t>
-  </si>
-  <si>
-    <t>Laboratorios Patagonia</t>
-  </si>
-  <si>
-    <t>Laboratorios Aconcagua</t>
-  </si>
-  <si>
-    <t>Laboratorios Iberá</t>
-  </si>
-  <si>
-    <t>Laboratorios Mitre</t>
-  </si>
-  <si>
-    <t>Farmacéutica Belgrano</t>
-  </si>
-  <si>
-    <t>Farmacéutica del Sur</t>
-  </si>
-  <si>
-    <t>Farmacéutica Rivadavia</t>
-  </si>
-  <si>
-    <t>Farmacéutica Costanera</t>
-  </si>
-  <si>
-    <t>Biogénesis Pharma</t>
-  </si>
-  <si>
-    <t>Genfar Argentina</t>
-  </si>
-  <si>
-    <t>Quimfarma</t>
-  </si>
-  <si>
-    <t>Medipharma SA</t>
-  </si>
-  <si>
-    <t>Innofarma</t>
-  </si>
-  <si>
-    <t>Prontosalud Labs</t>
-  </si>
-  <si>
-    <t>Droguería del Centro</t>
-  </si>
-  <si>
-    <t>Droguería La Estrella</t>
-  </si>
-  <si>
-    <t>Droguería San Martín</t>
-  </si>
-  <si>
-    <t>Droguería del Litoral</t>
-  </si>
-  <si>
-    <t>Droguería Continental</t>
-  </si>
-  <si>
-    <t>Dermalia Cosmética</t>
-  </si>
-  <si>
-    <t>Dermosur</t>
-  </si>
-  <si>
-    <t>Piel &amp; Sol Dermocosmética</t>
-  </si>
-  <si>
-    <t>Belladerm</t>
-  </si>
-  <si>
-    <t>Rostro Puro</t>
-  </si>
-  <si>
-    <t>Esencia Vital Perfumería</t>
-  </si>
-  <si>
-    <t>Aromas del Plata</t>
-  </si>
-  <si>
-    <t>Perfumería Alameda</t>
-  </si>
-  <si>
-    <t>Nutrivida Suplementos</t>
-  </si>
-  <si>
-    <t>Fortex Nutrition</t>
-  </si>
-  <si>
-    <t>ProteoLab Deportes</t>
-  </si>
-  <si>
-    <t>Vitalfar Suplementos</t>
-  </si>
-  <si>
-    <t>Omega Natural</t>
-  </si>
-  <si>
-    <t>Herbolaria Andina</t>
-  </si>
-  <si>
-    <t>Naturalis Fitoterapia</t>
-  </si>
-  <si>
-    <t>Kindel Bebés</t>
-  </si>
-  <si>
-    <t>Mamá &amp; Bebé SRL</t>
-  </si>
-  <si>
-    <t>Pequeños Pasos Infantil</t>
-  </si>
-  <si>
-    <t>Nutribaby Argentina</t>
-  </si>
-  <si>
-    <t>Sanix Descartables</t>
-  </si>
-  <si>
-    <t>Insumed Hospitalario</t>
-  </si>
-  <si>
-    <t>Botiquín Express</t>
-  </si>
-  <si>
-    <t>Primeros Auxilios SA</t>
-  </si>
-  <si>
-    <t>TecnoSalud Equipamiento</t>
-  </si>
-  <si>
-    <t>OptiVisión Óptica</t>
-  </si>
-  <si>
-    <t>Lentes del Sol SA</t>
-  </si>
-  <si>
-    <t>Audiofarma</t>
-  </si>
-  <si>
-    <t>Ortopedia Movilidad</t>
-  </si>
-  <si>
-    <t>Cuidado Mayor SRL</t>
-  </si>
-  <si>
-    <t>Higial Higiene</t>
-  </si>
-  <si>
-    <t>Blancaflor Tocador</t>
-  </si>
-  <si>
-    <t>Aquavital Cuidado Personal</t>
-  </si>
-  <si>
-    <t>Puravit Wellness</t>
-  </si>
-  <si>
-    <t>Farmax Genéricos</t>
-  </si>
-  <si>
-    <t>Curapel Dermatología</t>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Vamma / Bioderma</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Dorothy Gray</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Algabo</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Parallel (Chicco-Avent)</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Beauty Solutions / Disney</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Bagó</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Cuenca</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Beauty Solutions / Oreiro</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Loval</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Combe</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Caviahue</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Johnson Family</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Comimpar</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Active Cosmetic</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>Ayudín</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Eurolab / Viasek</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>Bernabó</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>Laboratorios ENA</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Elea / Adermicin</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>IDI</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Genoma</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Improm (Contigo / Nuk)</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>SISCOM</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Plumari / Estereocolor</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>Ferrini / Max</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>Buhl</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>ACF</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>Lancôme</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Biosintex</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Loreal / Dermo</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>BIC</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>Cdimex</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>Nestlé</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>Procter</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>Unilever Limpieza / Ala</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>Unilever Capilar / Sedal</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Biferdil</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>Kimberly</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>Cannon</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>Coty</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>Colgate</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>By Derm / Star</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>Essity</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>Loreal / Maquillajes</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>Unilever Rexona</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>Nivea / Eucerin</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>Johnson / Neutrogena</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>Papelera</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Andrómaco</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>Farmar</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>Facor</t>
   </si>
 </sst>
 </file>
@@ -573,7 +702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -585,483 +714,419 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
+      <c r="A3" t="s">
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
+      <c r="A4" t="s">
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
+      <c r="A5" t="s">
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
+      <c r="A6" t="s">
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
+      <c r="A7" t="s">
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
+      <c r="A8" t="s">
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
+      <c r="A9" t="s">
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
+      <c r="A10" t="s">
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
+      <c r="A11" t="s">
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
+      <c r="A12" t="s">
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
+      <c r="A13" t="s">
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
+      <c r="A14" t="s">
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
+      <c r="A15" t="s">
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
+      <c r="A16" t="s">
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
+      <c r="A17" t="s">
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>17</v>
+      <c r="A18" t="s">
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>18</v>
+      <c r="A19" t="s">
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
+      <c r="A20" t="s">
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
+      <c r="A21" t="s">
+        <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
+      <c r="A22" t="s">
+        <v>41</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
+      <c r="A23" t="s">
+        <v>43</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>23</v>
+      <c r="A24" t="s">
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>24</v>
+      <c r="A25" t="s">
+        <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
+      <c r="A26" t="s">
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>26</v>
+      <c r="A27" t="s">
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>27</v>
+      <c r="A28" t="s">
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>28</v>
+      <c r="A29" t="s">
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>29</v>
+      <c r="A30" t="s">
+        <v>57</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>30</v>
+      <c r="A31" t="s">
+        <v>59</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>31</v>
+      <c r="A32" t="s">
+        <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>32</v>
+      <c r="A33" t="s">
+        <v>63</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>33</v>
+      <c r="A34" t="s">
+        <v>65</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>34</v>
+      <c r="A35" t="s">
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>35</v>
+      <c r="A36" t="s">
+        <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>36</v>
+      <c r="A37" t="s">
+        <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>37</v>
+      <c r="A38" t="s">
+        <v>73</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>38</v>
+      <c r="A39" t="s">
+        <v>75</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>39</v>
+      <c r="A40" t="s">
+        <v>77</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>40</v>
+      <c r="A41" t="s">
+        <v>79</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>41</v>
+      <c r="A42" t="s">
+        <v>81</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>42</v>
+      <c r="A43" t="s">
+        <v>83</v>
       </c>
       <c r="B43" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>43</v>
+      <c r="A44" t="s">
+        <v>85</v>
       </c>
       <c r="B44" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>44</v>
+      <c r="A45" t="s">
+        <v>87</v>
       </c>
       <c r="B45" t="s">
-        <v>45</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>45</v>
+      <c r="A46" t="s">
+        <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47">
-        <v>46</v>
+      <c r="A47" t="s">
+        <v>91</v>
       </c>
       <c r="B47" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>47</v>
+      <c r="A48" t="s">
+        <v>93</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>48</v>
+      <c r="A49" t="s">
+        <v>95</v>
       </c>
       <c r="B49" t="s">
-        <v>49</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>49</v>
+      <c r="A50" t="s">
+        <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>50</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>50</v>
+      <c r="A51" t="s">
+        <v>99</v>
       </c>
       <c r="B51" t="s">
-        <v>51</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>51</v>
+      <c r="A52" t="s">
+        <v>101</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>52</v>
+      <c r="A53" t="s">
+        <v>103</v>
       </c>
       <c r="B53" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>54</v>
-      </c>
-      <c r="B55" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>55</v>
-      </c>
-      <c r="B56" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>56</v>
-      </c>
-      <c r="B57" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59">
-        <v>58</v>
-      </c>
-      <c r="B59" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60">
-        <v>59</v>
-      </c>
-      <c r="B60" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61">
-        <v>60</v>
-      </c>
-      <c r="B61" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>